<commit_message>
add a field validation in click method
</commit_message>
<xml_diff>
--- a/src/test/resources/Database/ruleData.xlsx
+++ b/src/test/resources/Database/ruleData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automation\ICEDQ-TestGenerator\src\test\resources\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3C73B33-1C25-4590-BC6C-455446841E06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED5D4BC2-9FF3-406F-82AC-7D2FD8896788}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dynamic Template" sheetId="1" r:id="rId1"/>
@@ -189,12 +189,6 @@
     <t>Redshift-without-jdbc-UserConn</t>
   </si>
   <si>
-    <t>7-8-0</t>
-  </si>
-  <si>
-    <t>7-8-0_Workflow</t>
-  </si>
-  <si>
     <t>Quality_Assurance</t>
   </si>
   <si>
@@ -202,6 +196,12 @@
   </si>
   <si>
     <t>FlatFile-SQL_Azure_Location_Azure_Access_Key--UserConn</t>
+  </si>
+  <si>
+    <t>7-9-4_Workflow</t>
+  </si>
+  <si>
+    <t>7-9-4</t>
   </si>
 </sst>
 </file>
@@ -621,7 +621,7 @@
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>21</v>
@@ -642,7 +642,7 @@
         <v>29</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="L2" t="s">
         <v>50</v>
@@ -659,7 +659,7 @@
         <v>8</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>21</v>
@@ -680,7 +680,7 @@
         <v>30</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="L3" t="s">
         <v>50</v>
@@ -697,7 +697,7 @@
         <v>8</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>21</v>
@@ -718,7 +718,7 @@
         <v>31</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="L4" t="s">
         <v>50</v>
@@ -735,7 +735,7 @@
         <v>8</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>21</v>
@@ -756,7 +756,7 @@
         <v>32</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="L5" t="s">
         <v>50</v>
@@ -773,7 +773,7 @@
         <v>8</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>22</v>
@@ -794,7 +794,7 @@
         <v>33</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="L6" t="s">
         <v>50</v>
@@ -811,7 +811,7 @@
         <v>8</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>22</v>
@@ -832,7 +832,7 @@
         <v>34</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="L7" t="s">
         <v>50</v>
@@ -849,7 +849,7 @@
         <v>8</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>22</v>
@@ -870,7 +870,7 @@
         <v>35</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="L8" t="s">
         <v>50</v>
@@ -887,7 +887,7 @@
         <v>8</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>22</v>
@@ -908,7 +908,7 @@
         <v>36</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="L9" t="s">
         <v>50</v>
@@ -976,7 +976,7 @@
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>21</v>
@@ -989,7 +989,7 @@
         <v>51</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
@@ -1003,7 +1003,7 @@
         <v>8</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>21</v>
@@ -1016,7 +1016,7 @@
         <v>51</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -1030,7 +1030,7 @@
         <v>8</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>21</v>
@@ -1043,7 +1043,7 @@
         <v>37</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -1057,7 +1057,7 @@
         <v>8</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>21</v>
@@ -1070,7 +1070,7 @@
         <v>37</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
@@ -1084,7 +1084,7 @@
         <v>8</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>21</v>
@@ -1097,7 +1097,7 @@
         <v>37</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
@@ -1111,7 +1111,7 @@
         <v>8</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>22</v>
@@ -1124,7 +1124,7 @@
         <v>52</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
@@ -1138,7 +1138,7 @@
         <v>8</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>22</v>
@@ -1151,7 +1151,7 @@
         <v>52</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
@@ -1165,7 +1165,7 @@
         <v>8</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>22</v>
@@ -1178,7 +1178,7 @@
         <v>27</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
@@ -1192,7 +1192,7 @@
         <v>8</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>22</v>
@@ -1205,7 +1205,7 @@
         <v>27</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
@@ -1219,7 +1219,7 @@
         <v>8</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>24</v>
@@ -1231,10 +1231,10 @@
         <v>45</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
@@ -1248,7 +1248,7 @@
         <v>8</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>24</v>
@@ -1260,10 +1260,10 @@
         <v>45</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
@@ -1277,7 +1277,7 @@
         <v>8</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>24</v>
@@ -1292,7 +1292,7 @@
         <v>45</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
@@ -1306,7 +1306,7 @@
         <v>8</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>24</v>
@@ -1321,10 +1321,10 @@
         <v>45</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>6</v>
       </c>
@@ -1335,7 +1335,7 @@
         <v>8</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>24</v>
@@ -1347,13 +1347,13 @@
         <v>41</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>10</v>
       </c>
@@ -1364,7 +1364,7 @@
         <v>8</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>24</v>
@@ -1376,10 +1376,10 @@
         <v>41</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
@@ -1393,7 +1393,7 @@
         <v>8</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>24</v>
@@ -1408,7 +1408,7 @@
         <v>41</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
@@ -1422,7 +1422,7 @@
         <v>8</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E18" s="5" t="s">
         <v>24</v>
@@ -1437,7 +1437,7 @@
         <v>41</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -1513,7 +1513,7 @@
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>21</v>
@@ -1534,7 +1534,7 @@
         <v>40</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="L2" t="s">
         <v>50</v>
@@ -1602,7 +1602,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
@@ -1613,7 +1613,7 @@
         <v>8</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>21</v>
@@ -1634,7 +1634,7 @@
         <v>40</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="L2" t="s">
         <v>50</v>

</xml_diff>